<commit_message>
feat: add row-level threat context to all controls
</commit_message>
<xml_diff>
--- a/generated/checklists/product-security-assessment-template.xlsx
+++ b/generated/checklists/product-security-assessment-template.xlsx
@@ -450,17 +450,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious or compromised dependency executing inside the build</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dependency code reads credentials or uses control-plane write access to alter repositories releases or infrastructure</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">removing credentials and write authority limits impact even when untrusted build code executes</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -637,17 +637,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised build process attempting to cross into deployment authority</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the environment executing dependencies also holds release or production deployment credentials</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an artifact-only handoff prevents build-time code from directly exercising deploy privileges</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious dependency or build script using outbound network access</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">build code exfiltrates source or downloads an unreviewed secondary payload from arbitrary destinations</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">default-deny egress constrains exfiltration and payload retrieval independently of filesystem controls</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">untrusted package build logic and compromised build tools</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">build code persists changes escalates through root privileges or writes outside the intended workspace</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ephemeral non-root read-only isolation reduces persistence and host compromise when execution is unavoidable</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1198,17 +1198,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious build code hiding activity within otherwise successful output</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unexpected processes or network connections occur without evidence for detection or incident reconstruction</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">containment reduces capability but telemetry is needed to detect attempts and verify boundary operation</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malformed evidence missing input or an operator misreading verifier failure</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">policy evaluation cannot complete but the build is reported as satisfying containment requirements</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a distinct error state prevents unavailable verification from becoming false assurance</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1572,17 +1572,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">producer selecting an unsuitable platform or a platform overstating guarantees</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">releases use a builder that cannot provide the hosted control and evidence required by the target level</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">platform capability must be approved before individual build records become meaningful evidence</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1759,17 +1759,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">developer or attacker substituting an unapproved local or tenant-controlled build</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a release artifact is produced outside the approved hosted builder while retaining a plausible record</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact builder identity ties every release to the assessed platform rather than a preferred process</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1946,17 +1946,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor or compromised pipeline changing build instructions independently of reviewed source</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the artifact is built with mutable or untraceable instructions differing from the reviewed revision</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">binding definition path and full revision makes the build process reviewable and repeatable</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unauthorized caller or pipeline drift altering parameters entry points or triggers</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the approved definition runs with unexpected inputs and produces a materially different artifact</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">definition identity alone does not constrain runtime invocation so parameters and trigger must also match</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -2320,17 +2320,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">incomplete build records malformed policy or verification infrastructure failure</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">consistency and hosted execution cannot be established but are recorded as passing</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">fail-closed verification keeps missing evidence distinct from an approved hosted build</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tenant build step disabling provenance or generating evidence only for selected builds</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a successful build completes without platform evidence or emits tenant-generated substitute metadata</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">mandatory automatic generation keeps provenance coverage outside the untrusted workload</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">artifact substituter or producer presenting provenance for a different output</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">valid-looking provenance does not identify the distributed artifact source or invocation</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">subject digest and build inputs establish what the evidence actually describes</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious tenant workload supplying false builder source or invocation fields</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker-controlled build steps claim a trusted builder identity or benign parameters</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">security-relevant fields must originate from the control plane rather than the workload they attest to</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -3068,17 +3068,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tenant build step or external party forging platform provenance</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">provenance is altered or newly signed using an identity available to untrusted workload code</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a platform-exclusive signing identity authenticates the evidence source and integrity</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -3255,17 +3255,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malformed provenance unavailable crypto tooling or operator error</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">signature or field validation does not complete but provenance is accepted</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">cryptographic assurance exists only after successful verification so tool and parse failures must block</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -3442,17 +3442,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised Action maintainer or attacker moving a mutable upstream ref</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a reviewed workflow later executes different third-party Action code without repository change</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a full commit SHA makes dependency updates explicit and reviewable in the consuming repository</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -3629,17 +3629,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised reusable-workflow provider changing a branch or tag</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">caller jobs inherit altered commands permissions or secret handling from an external workflow</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">reusable workflows execute substantial remote policy and therefore need the same immutable binding as Actions</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -3816,17 +3816,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">container publisher or registry attacker replacing a mutable Action image tag</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Docker-based Action pulls different bytes while its tag and workflow text remain unchanged</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an image digest binds execution to exact container content instead of a mutable registry label</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -4003,17 +4003,17 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor introducing a tag branch short SHA or computed external reference</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">workflow review cannot determine the exact third-party code that will execute</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">rejecting every mutable and dynamic form closes bypasses left by checking only common Action syntax</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -4190,17 +4190,17 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malformed workflow unsupported syntax or failed reference parser</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the verifier cannot inspect a dependency reference but reports no mutable references</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">parser and execution errors must remain distinct so incomplete inspection never appears compliant</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -4377,17 +4377,17 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pull-request author controlling branch issue label commit or event data</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an Actions expression is substituted directly into a generated shell script and becomes executable syntax</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">excluding expressions from run scalars removes the code-generation boundary where data becomes commands</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -4564,17 +4564,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">untrusted contributor crafting shell metacharacters in workflow context values</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker-controlled text crosses into shell execution without a data boundary or safe quoting</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">environment variables preserve the value as data and allow shell-specific quoting at the consumption point</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">benign workflow author using expressions in declarative non-shell fields</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">context-insensitive scanning blocks safe metadata and creates noise that encourages disabling the control</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">limiting findings to executable fields preserves signal and makes enforcement operationally sustainable</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -4938,17 +4938,17 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malformed or unsupported YAML hiding executable content from analysis</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">parser failure is interpreted as no direct interpolation and the workflow is accepted</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">explicit ERROR prevents syntactic ambiguity from bypassing command-injection checks</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -5125,17 +5125,17 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised scanner publisher or mutable Action reference</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the security job silently runs different analysis code or rules than reviewers approved</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pinned scanner and Action identities make the verifier itself a controlled supply-chain dependency</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -5312,17 +5312,17 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious pull-request author whose workflow content is scanned</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">untrusted PR input executes in a scanner job holding write tokens or privileged credentials</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">credential-free gating detects workflow weaknesses without turning analysis into a secret-exfiltration path</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -5499,17 +5499,17 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">untrusted pull request attempting to misuse SARIF upload authority</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">security-events write permission is exposed to fork-controlled code or events</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">separating trusted upload from untrusted gating preserves reporting without granting PRs privileged API access</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -5686,17 +5686,17 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">scanner crash malformed SARIF or operator confusing execution failure with zero findings</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">analysis does not complete but the workflow receives a successful clean result</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">distinct clean finding and error states preserve fail-closed enforcement and trustworthy metrics</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -5873,17 +5873,17 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor weakening permissions events or scanner arguments after initial adoption</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the deployed workflow drifts from the reviewed sample while local fixtures continue to pass</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">baseline comparison verifies the actual adopted workflow rather than only the reference implementation</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -6060,17 +6060,17 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker publishing a compromised package version through a maintainer account</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">automation adopts the release immediately before community detection yanking or advisory publication</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a minimum observation window reduces exposure to attacks whose warning signals emerge shortly after release</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -6247,17 +6247,17 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">maintainer bypassing cooldown for urgent fixes or attacker abusing a broad exception</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an exception covers extra packages versions or time beyond the reviewed emergency</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact owned expiring approval permits urgent response without permanently removing the observation window</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -6434,17 +6434,17 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">configuration drift or contributor reducing the waiting period for convenience</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">nominal cooldown remains enabled but its value is lowered below the reviewed baseline</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">enforcing the policy floor prevents semantic weakening that a simple enabled check would miss</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -6621,17 +6621,17 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dependency-confusion publisher or registry metadata source controlled by an attacker</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">release age and version facts come from an unapproved registry origin</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">cooldown decisions are trustworthy only when metadata is bound to an approved credential-free HTTPS source</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -6808,17 +6808,17 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">metadata tampering cache poisoning or artifact replacement after age approval</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an old enough version passes cooldown but its metadata or downloaded bytes differ from expected content</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integrity checks ensure cooldown applies to the exact artifact under review rather than only its version label</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -6995,17 +6995,17 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">registry failure malformed metadata missing artifact or assessment tooling error</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">release age or integrity cannot be established but dependency adoption is reported clean</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">operational failure must block or escalate because no observation guarantee was verified</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -7182,17 +7182,17 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious npm or Bun package publishing lifecycle scripts</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">install automatically executes dependency-controlled code with developer or CI privileges</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">repository-owned default deny removes the most common implicit execution path before package use</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -7369,17 +7369,17 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised pnpm dependency requesting a native or lifecycle build</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">broad or permanent build approval lets unreviewed package versions execute during install</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact time-bound approval limits execution to the reviewed package need and forces reevaluation</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -7556,17 +7556,17 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious Python source distribution or compromised build backend</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pip falls back to source build and executes backend code not represented by the expected wheel</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">binary-only exact hashes bind installation to reviewed artifacts and avoid source-build execution</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -7743,17 +7743,17 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">maintainer creating an overly broad exception to resolve installation friction</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">wildcard package approval or expired justification becomes a permanent arbitrary-code path</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">narrow owned expiring exceptions preserve default deny while allowing explicitly reviewed necessity</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -7930,17 +7930,17 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">missing malformed or unsupported package-manager configuration</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">install execution policy cannot be evaluated but is reported as safely disabled</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a distinct error prevents configuration absence from becoming silent permission to execute</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -8117,17 +8117,17 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor or tooling changing dependencies without regenerating reviewed lock state</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">manifest intent and installed exact graph diverge so reviewers assess different dependencies than builds use</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">graph equality makes the lockfile a faithful executable representation of the reviewed manifest</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -8304,17 +8304,17 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dependency-confusion publisher network attacker or credential-bearing registry misconfiguration</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">packages resolve from an unapproved origin or registry access leaks credentials</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a credential-free HTTPS origin allowlist constrains both package source and transport trust</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -8491,17 +8491,17 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">registry compromise cache poisoning or artifact substitution in transit</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the resolved package name and version are correct but downloaded bytes differ from reviewed content</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">artifact digest verification protects the content boundary that version pinning alone cannot</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -8678,17 +8678,17 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor introducing ranges floating selectors or implicit lockfile updates</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">future resolution changes the dependency graph without a corresponding reviewed repository diff</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact frozen resolution makes dependency changes explicit and reproducible</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -8865,17 +8865,17 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unreadable malformed or missing manifest lockfile metadata or artifact</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integrity comparison cannot complete yet reports a clean dependency graph</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ERROR state preserves the difference between verified equality and unavailable evidence</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -9052,17 +9052,17 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised dependency maintainer or attacker introducing a malicious exact package version</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">responders know the package version but cannot identify affected repositories builds and artifacts</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact reverse lookup converts a dependency alert into an actionable and bounded incident scope</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -9239,17 +9239,17 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">stale inventory tampering or accidental mismatch between SBOM and build records</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">response decisions use an SBOM that does not correspond to the investigated build or evidence artifact</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integrity links establish that inventory findings refer to the actual product build under investigation</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -9426,17 +9426,17 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">rushed responder or unauthorized automation performing destructive containment</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">caches credentials or artifacts are removed before evidence capture causing investigation loss or outage</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">preservation-first owner-approved dry runs make response actions reviewable before changing production state</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -9613,17 +9613,17 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">incomplete assessment tooling or responder misinterpreting no result as no impact</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">impacted no-impact and verification-failure outcomes collapse into one ambiguous status</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">distinct states determine whether to contain close or repair the assessment rather than guess</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -9800,17 +9800,17 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">incomplete asset inventory unsafe runbook or unreviewed response configuration</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">response proceeds while products are missing from scope or destructive steps lack safeguards</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">validation blocks plans that could miss affected assets or damage evidence and availability</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -9987,17 +9987,17 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker substituting an artifact while reusing unrelated valid provenance</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">downloaded bytes differ from the subject digest authenticated by provenance</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">signature validity alone does not bind evidence to the exact artifact being consumed</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -10174,17 +10174,17 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">external forger or unauthorized signer creating plausible provenance</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">provenance content is modified or signed by an identity the consumer did not approve</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">consumer-owned trust roots authenticate provenance origin and integrity before field evaluation</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -10361,17 +10361,17 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised builder producer or release channel presenting authentic but unexpected output</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">correctly signed provenance names an unapproved builder source revision ref or build type</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">authenticity does not establish policy acceptability so consumer expectations must be checked separately</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -10548,17 +10548,17 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">release operator or attacker removing verification signals to bypass a failing check</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a previously protected artifact family is distributed without required signature or provenance</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">explicit no-downgrade rules prevent absence of evidence from silently becoming an accepted legacy path</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -10735,17 +10735,17 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malformed input unavailable cryptographic tooling or verifier infrastructure failure</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">authenticity cannot be evaluated but the release is reported as trusted</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a separate error state ensures operational failure never becomes a clean verification result</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -10922,17 +10922,17 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malware credential stealer or attacker obtaining cached developer credentials</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a long-lived token remains usable after theft and grants sustained source or service access</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">short-lived sessions reduce the exploitation window independently of endpoint detection and revocation speed</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -11109,17 +11109,17 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">local malware another user or accidental file disclosure</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">plaintext credential files or Git helpers expose reusable secrets from developer storage</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an approved OS-backed store adds access control and avoids recoverable plaintext persistence</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -11296,17 +11296,17 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malware or attacker attempting to copy a developer private key</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an exportable key is stolen and used from another device without user verification</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">hardware-backed non-exportable keys constrain credential use even after filesystem compromise</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -11483,17 +11483,17 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">developer accidentally staging a secret or malware placing one in the worktree</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">sensitive content enters a commit before repository-side controls can react</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pre-commit scanning provides immediate prevention at the earliest source-publication boundary</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -11670,17 +11670,17 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor bypassing local hooks Web UI user or unmanaged clone</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a secret reaches the shared repository through a path where endpoint scanning did not run</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">mandatory server-side enforcement covers publication paths and bypasses outside local policy</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -11857,17 +11857,17 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious package install script or compromised build backend</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dependency installation reads developer files credentials sockets or modifies the host</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">disposable restricted installation isolates unavoidable package execution from endpoint assets</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -12044,17 +12044,17 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker publishing a new compromised dependency or maintainer delaying an urgent security fix</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">automation adopts a fresh malicious release or cooldown blocks necessary remediation without review</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">cooldown plus narrow security exception balances observation time with controlled urgent updates</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -12231,17 +12231,17 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malware malicious development tool or compromised dependency using outbound connectivity</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">source credentials or prompts are exfiltrated to an arbitrary external endpoint</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">managed destination allowlisting limits exfiltration when local process controls are bypassed</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -12418,17 +12418,17 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">phishing adversary or attacker using an orphaned developer account</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">stolen passwords or incomplete offboarding grant repository and development-service access</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">centralized lifecycle and phishing-resistant MFA address identity compromise beyond device configuration</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -12605,17 +12605,17 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">developer or tool adding archives databases keys binaries or oversized sensitive files</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">high-risk file types bypass text-only secret patterns and enter source history</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">file type size and content guards cover disclosure forms that credential regex alone cannot</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -12792,17 +12792,17 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">thief or unauthorized person obtaining a powered-off developer device or storage media</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">source credentials caches and local artifacts are read directly from unencrypted storage</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">full-disk encryption protects data at rest when login and runtime controls are unavailable</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -12979,17 +12979,17 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">nearby unauthorized person accessing an unattended unlocked workstation</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an active developer session exposes source credentials and authenticated services without device theft</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">enforced inactivity lock shortens physical access opportunity during routine absence</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -13166,17 +13166,17 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker exploiting known vulnerabilities in the OS browser editor or developer tools</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unsupported or unpatched software enables local compromise and credential theft</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">automatic enforced security updates reduce exposure time to publicly known endpoint exploits</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -13353,17 +13353,17 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious package tool or user mistake executing with administrator authority</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">routine development code modifies system security settings credentials or other users data</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">standard-user operation limits blast radius while controlled elevation preserves necessary administration</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -13540,17 +13540,17 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malware backup process support tool or accidental repository publication</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">credentials stored in workspaces dotfiles or shell history are copied or committed</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">absence checks address secret locations outside approved stores that secure-helper configuration does not cover</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -13727,17 +13727,17 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised container dependency or development tool accessing the host runtime socket</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unrestricted Docker socket access becomes effective root-level control of the endpoint</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">removing broad socket access preserves the container boundary instead of exposing a host takeover interface</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -13914,17 +13914,17 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">network attacker discovering an unmanaged debugger database or development service</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a debug listener exposes code execution data or unauthenticated administration beyond loopback</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">default-disabled externally reachable services reduce attack surface not covered by repository controls</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -14101,17 +14101,17 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised AI tool MCP server plugin or malicious prompt causing unauthorized network access</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">source prompts credentials or workspace data are sent to unapproved services</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">destination controls bound AI integrations whose dynamic behavior may exceed the immediate coding task</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -14288,17 +14288,17 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compromised sandbox process package or AI agent with mounted host paths</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">development workload overwrites source credentials configuration or unrelated host files</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">read-only defaults make write authority explicit and narrow rather than inheriting the whole workspace</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -14475,17 +14475,17 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">backup service compromise storage theft or unauthorized backup administrator</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">historical source credentials and local artifacts remain readable in backup copies</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">encrypted access-controlled backups extend endpoint confidentiality to retained copies and recovery media</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -14662,17 +14662,17 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker or compromised shared filesystem replacing executable Git hooks</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a commit or push silently runs unreviewed code outside the repository security review boundary</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">repository-relative reviewed hooks make the executed prevention logic visible and governable</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -14849,17 +14849,17 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">local attacker installer or stale global configuration redirecting hook execution</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Git loads hooks from an absolute shared or globally managed path that repository reviewers cannot inspect</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">rejecting external hook paths prevents repository policy from being substituted at runtime</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -15036,17 +15036,17 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malware local user backup process or accidental remote URL disclosure</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Git stores reusable credentials in plaintext or embeds them in repository configuration</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">approved helpers and credential-free URLs remove persistent secrets outside content scanning coverage</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -15223,17 +15223,17 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker controlling a repository owned by another local account</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">wildcard safe.directory causes Git to trust ownership-unsafe worktrees and execute their configuration</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact trusted paths preserve Git ownership checks instead of disabling them globally</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -15410,17 +15410,17 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">impersonating contributor or user accidentally pushing more refs than intended</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unsigned history obscures author identity or broad push defaults publish unrelated branches and tags</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">signing and narrow push behavior protect identity and publication scope beyond content scanning</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -15597,17 +15597,17 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">developer tool or malware adding binaries archives databases key stores or sensitive metadata</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dangerous non-text content enters Git while evading ordinary secret regex review</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">explicit file-format denial covers opaque and high-risk artifacts that content patterns cannot reliably inspect</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -15784,17 +15784,17 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">accidental contributor or malware placing credential-like content in a file</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">supported secret patterns are committed and scanner output further leaks the matched value</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">detection with redacted reporting blocks representative credentials without creating a second disclosure channel</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -15971,17 +15971,17 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">user or tool adding a large opaque file that exceeds local review and scanner limits</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">sensitive content hides in an oversized file that is skipped for performance</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">rejecting rather than skipping enforces an explicit artifact-storage decision and prevents an unscanned gap</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -16158,17 +16158,17 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor accidentally staging a sensitive file or credential</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">content reaches immutable local history before the developer receives feedback</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">index scanning acts at the earliest exact commit boundary and avoids scanning unrelated working-tree state</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -16345,17 +16345,17 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor copying a token internal URL or sensitive text into a commit message</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">metadata becomes permanently searchable even when all committed files are clean</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">commit messages are a separate Git publication surface not inspected by staged-file scanning</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -16532,17 +16532,17 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor bypassing commit hooks then deleting the secret in a later commit</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">latest tree is clean but the pushed range introduces an earlier recoverable secret</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pre-push range scanning covers every introduced commit and closes latest-state and no-verify bypasses</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -16719,17 +16719,17 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">missing Git scanner crash malformed input or operator treating hook failure as success</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the operation proceeds because inspection could not run rather than because content was clean</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">distinct fail-closed errors preserve the security meaning of a zero-finding result</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -16906,17 +16906,17 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">configuration drift mutable external hook or incomplete pre-commit installation</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">framework adoption omits commit-message or push-history checks or downloads changing hook code</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">reviewed three-stage repository-owned configuration preserves native control coverage under the alternate framework</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -17093,17 +17093,17 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">credential exposure outside the repository-owned scanner rule set or compromised mutable scanner source</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a secret pattern is missed by one engine or scanner output and installation drift weaken detection</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">an independently pinned redacted Gitleaks scan adds rule diversity while retaining controlled execution</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -35836,17 +35836,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">producer selecting an unsuitable platform or a platform overstating guarantees</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">releases use a builder that cannot provide the hosted control and evidence required by the target level</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">platform capability must be approved before individual build records become meaningful evidence</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -36023,17 +36023,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">developer or attacker substituting an unapproved local or tenant-controlled build</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a release artifact is produced outside the approved hosted builder while retaining a plausible record</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">exact builder identity ties every release to the assessed platform rather than a preferred process</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -36210,17 +36210,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">contributor or compromised pipeline changing build instructions independently of reviewed source</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the artifact is built with mutable or untraceable instructions differing from the reviewed revision</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">binding definition path and full revision makes the build process reviewable and repeatable</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -36397,17 +36397,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">unauthorized caller or pipeline drift altering parameters entry points or triggers</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">the approved definition runs with unexpected inputs and produces a materially different artifact</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">definition identity alone does not constrain runtime invocation so parameters and trigger must also match</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -36584,17 +36584,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tenant build step disabling provenance or generating evidence only for selected builds</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a successful build completes without platform evidence or emits tenant-generated substitute metadata</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">mandatory automatic generation keeps provenance coverage outside the untrusted workload</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -36771,17 +36771,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">artifact substituter or producer presenting provenance for a different output</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">valid-looking provenance does not identify the distributed artifact source or invocation</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">subject digest and build inputs establish what the evidence actually describes</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -36958,17 +36958,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">malicious tenant workload supplying false builder source or invocation fields</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker-controlled build steps claim a trusted builder identity or benign parameters</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">security-relevant fields must originate from the control plane rather than the workload they attest to</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -37145,17 +37145,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tenant build step or external party forging platform provenance</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">provenance is altered or newly signed using an identity available to untrusted workload code</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">a platform-exclusive signing identity authenticates the evidence source and integrity</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -37332,17 +37332,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">attacker substituting an artifact while reusing unrelated valid provenance</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">downloaded bytes differ from the subject digest authenticated by provenance</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">signature validity alone does not bind evidence to the exact artifact being consumed</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -37519,17 +37519,17 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">external forger or unauthorized signer creating plausible provenance</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">provenance content is modified or signed by an identity the consumer did not approve</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">consumer-owned trust roots authenticate provenance origin and integrity before field evaluation</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">

</xml_diff>